<commit_message>
Add honest active-learning depth fields and friendly step-label support
Wire the deterministic time-depth estimator into the canonical time model so
every card/lesson/module carries an honest (no-double-count) active-learning
estimate, a content_depth_gap_minutes, and an under_depth flag. The 720-minute
syllabus allocation is preserved (not recomputed); gaps are reported, not padded.

Regenerate all mirrored artifacts from canonical JSON. Refresh the time-depth
audit (qa/): ~426.6 active min (~7.1 h) vs 720 declared; M01-M06 flagged
under-depth for source-grounded expansion.

(Learner-facing flowchart friendly-label fix is applied in LessonPlayerPage but
left uncommitted because it is interwoven with the in-progress branding refactor.)

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/CNA-Recert-Course/ContentV2/xlsx/CNA_RECERT_CONTENTV2_MASTER.xlsx
+++ b/CNA-Recert-Course/ContentV2/xlsx/CNA_RECERT_CONTENTV2_MASTER.xlsx
@@ -592,7 +592,7 @@
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>authored</t>
+          <t>under-depth</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
@@ -643,7 +643,7 @@
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>authored-partial</t>
+          <t>under-depth</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
@@ -745,7 +745,7 @@
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>authored-partial</t>
+          <t>under-depth</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
@@ -796,7 +796,7 @@
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>authored-partial</t>
+          <t>under-depth</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
@@ -847,7 +847,7 @@
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>authored-partial</t>
+          <t>under-depth</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
@@ -36621,7 +36621,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>2026-06-02T00:31:57+00:00</t>
+          <t>2026-06-02T01:57:05+00:00</t>
         </is>
       </c>
     </row>

</xml_diff>